<commit_message>
test: expand cross-engine compatibility test suite coverage
- Upgraded the python (openpyxl) and go (excelize) fixture generator scripts to produce significantly more complex .xlsx files.
- The generated files now inject Date/Time strings, Mathematical Formulas (=SUM), Merged Cells, multi-axis Cell Borders, and Multiple Worksheets.
- Enhanced `testXLCompatibility.cpp` assertions to parse these advanced elements, ensuring OpenXLSX maintains lossless compatibility when opening, modifying, and saving structurally complex third-party sheets.
</commit_message>
<xml_diff>
--- a/Tests/Fixtures/excelize_generated.xlsx
+++ b/Tests/Fixtures/excelize_generated.xlsx
@@ -8,18 +8,25 @@
   </bookViews>
   <sheets>
     <sheet name="TestSheet" sheetId="1" r:id="rId1"/>
+    <sheet name="SecondSheet" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>Hello from excelize</t>
   </si>
   <si>
     <t>Styled</t>
+  </si>
+  <si>
+    <t>Merged Area</t>
+  </si>
+  <si>
+    <t>Data in second sheet</t>
   </si>
 </sst>
 </file>
@@ -34,8 +41,10 @@
       <sz val="11"/>
     </font>
     <font>
+      <name val="Comic Sans MS"/>
       <family val="2"/>
       <b val="1"/>
+      <i val="1"/>
       <color rgb="FFFF0000"/>
     </font>
   </fonts>
@@ -52,7 +61,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -60,14 +69,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="false">
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyAlignment="false">
       <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -343,8 +369,11 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="2">
@@ -357,6 +386,32 @@
         <v>3.1415</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="1">
+        <v>45440.604166666664</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <f>=SUM(A2:A3)</f>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C1:E2"/>
+  </mergeCells>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>